<commit_message>
feat(qa): save all Sprint 3 test cases, Store Locator map retest, and audit artifacts
</commit_message>
<xml_diff>
--- a/Sprint-3/Ticket_41794519_Homepage/Homepage_Test_Cases.xlsx
+++ b/Sprint-3/Ticket_41794519_Homepage/Homepage_Test_Cases.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="QA Test Cases" sheetId="1" r:id="rId1"/>
+    <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,19 +397,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:J16"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="18.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-    <col min="4" max="4" width="35.83203125" customWidth="1"/>
-    <col min="5" max="5" width="30.83203125" customWidth="1"/>
-    <col min="6" max="6" width="45.83203125" customWidth="1"/>
-    <col min="7" max="7" width="45.83203125" customWidth="1"/>
-    <col min="8" max="8" width="45.83203125" customWidth="1"/>
-    <col min="9" max="9" width="15.83203125" customWidth="1"/>
-    <col min="10" max="10" width="40.83203125" customWidth="1"/>
-    <col min="11" max="11" width="35.83203125" customWidth="1"/>
+    <col min="1" max="1" width="16.83203125" customWidth="1"/>
+    <col min="2" max="2" width="29.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="64.83203125" customWidth="1"/>
+    <col min="5" max="5" width="64.83203125" customWidth="1"/>
+    <col min="6" max="6" width="64.83203125" customWidth="1"/>
+    <col min="7" max="7" width="64.83203125" customWidth="1"/>
+    <col min="8" max="8" width="64.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="64.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -443,9 +442,6 @@
       <c r="J1" t="str">
         <v>Defect Summary</v>
       </c>
-      <c r="K1" t="str">
-        <v>Visual Evidence</v>
-      </c>
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
@@ -480,9 +476,6 @@
       <c r="J2" t="str">
         <v>None. Verified acceptable for staging environment.</v>
       </c>
-      <c r="K2" t="str">
-        <v>screenshots/desktop/01_desktop_homepage_full.png</v>
-      </c>
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3" t="str">
@@ -517,9 +510,6 @@
       <c r="J3" t="str">
         <v>None. Verified matching approved specification.</v>
       </c>
-      <c r="K3" t="str">
-        <v>screenshots/desktop/02_desktop_utility_bar.png</v>
-      </c>
     </row>
     <row r="4" xml:space="preserve">
       <c r="A4" t="str">
@@ -554,9 +544,6 @@
       <c r="J4" t="str">
         <v>None. Verified matching AU design baseline.</v>
       </c>
-      <c r="K4" t="str">
-        <v>comparison/COMPARISON_PASS_01_HERO_BANNER_SLIDER.png</v>
-      </c>
     </row>
     <row r="5" xml:space="preserve">
       <c r="A5" t="str">
@@ -591,9 +578,6 @@
       <c r="J5" t="str">
         <v>None. Previous Ticket 4 defect successfully resolved.</v>
       </c>
-      <c r="K5" t="str">
-        <v>screenshots/desktop/03_hero_banner_slider.png</v>
-      </c>
     </row>
     <row r="6" xml:space="preserve">
       <c r="A6" t="str">
@@ -628,9 +612,6 @@
       <c r="J6" t="str">
         <v>None. Verified matching AU design baseline.</v>
       </c>
-      <c r="K6" t="str">
-        <v>comparison/COMPARISON_PASS_02_CATEGORY_CAROUSEL.png</v>
-      </c>
     </row>
     <row r="7" xml:space="preserve">
       <c r="A7" t="str">
@@ -665,9 +646,6 @@
       <c r="J7" t="str">
         <v>None. Verified matching approved design baseline.</v>
       </c>
-      <c r="K7" t="str">
-        <v>screenshots/desktop/05_about_us_brand_story.png</v>
-      </c>
     </row>
     <row r="8" xml:space="preserve">
       <c r="A8" t="str">
@@ -702,9 +680,6 @@
       <c r="J8" t="str">
         <v>None. Verified matching approved design baseline.</v>
       </c>
-      <c r="K8" t="str">
-        <v>screenshots/desktop/06_b2b_video_block.png</v>
-      </c>
     </row>
     <row r="9" xml:space="preserve">
       <c r="A9" t="str">
@@ -739,9 +714,6 @@
       <c r="J9" t="str">
         <v>None. Manually verified passing by QA Lead.</v>
       </c>
-      <c r="K9" t="str">
-        <v>screenshots/desktop/07_recent_articles_journal.png</v>
-      </c>
     </row>
     <row r="10" xml:space="preserve">
       <c r="A10" t="str">
@@ -776,9 +748,6 @@
       <c r="J10" t="str">
         <v>None. Manually verified passing by QA Lead.</v>
       </c>
-      <c r="K10" t="str">
-        <v>screenshots/desktop/08_instagram_feed.png</v>
-      </c>
     </row>
     <row r="11" xml:space="preserve">
       <c r="A11" t="str">
@@ -813,9 +782,6 @@
       <c r="J11" t="str">
         <v>None. Verified matching approved design specification.</v>
       </c>
-      <c r="K11" t="str">
-        <v>screenshots/desktop/01_desktop_homepage_full.png</v>
-      </c>
     </row>
     <row r="12" xml:space="preserve">
       <c r="A12" t="str">
@@ -850,9 +816,6 @@
       <c r="J12" t="str">
         <v>Storefront footer "Shop Outlet" link leaks US buyers to external Australian website (https://globewestoutlet.com.au/).</v>
       </c>
-      <c r="K12" t="str">
-        <v>screenshots/defects/DEFECT_AU_OUTLET_URL_FOOTER_RED_BOX.png</v>
-      </c>
     </row>
     <row r="13" xml:space="preserve">
       <c r="A13" t="str">
@@ -887,9 +850,6 @@
       <c r="J13" t="str">
         <v>None. Verified passing mobile responsive standard.</v>
       </c>
-      <c r="K13" t="str">
-        <v>comparison/COMPARISON_PASS_04_MOBILE_RESPONSIVE.png</v>
-      </c>
     </row>
     <row r="14" xml:space="preserve">
       <c r="A14" t="str">
@@ -924,9 +884,6 @@
       <c r="J14" t="str">
         <v>None. Verified matching approved security and auth matrix.</v>
       </c>
-      <c r="K14" t="str">
-        <v>comparison/COMPARISON_PASS_03_DUAL_AUTH_MATRIX.png</v>
-      </c>
     </row>
     <row r="15" xml:space="preserve">
       <c r="A15" t="str">
@@ -961,9 +918,6 @@
       <c r="J15" t="str">
         <v>None. Verified matching approved trade portal specification.</v>
       </c>
-      <c r="K15" t="str">
-        <v>screenshots/desktop/10_authenticated_trade_homepage.png</v>
-      </c>
     </row>
     <row r="16" xml:space="preserve">
       <c r="A16" t="str">
@@ -982,7 +936,10 @@
         <v>Full homepage DOM loaded with AxeBuilder rulesets</v>
       </c>
       <c r="F16" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Run AxeBuilder against WCAG 2.0, 2.1, 2.2 Level A and AA rules
+        <v xml:space="preserve">1. Run AxeBuilder against WCAG
+2.0,
+2.1,
+2.2 Level A and AA rules
 2. Inspect for critical violations (contrast, alt text, ARIA roles, landmarks)</v>
       </c>
       <c r="G16" t="str">
@@ -997,13 +954,10 @@
       <c r="J16" t="str">
         <v>None. Passed Phase 1 accessibility gate.</v>
       </c>
-      <c r="K16" t="str">
-        <v>scripts/ticket_homepage_audit.spec.js</v>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>